<commit_message>
feat: authenticate relocated approval challenges with a vault origin key
Operators can copy a Broker-signed challenge envelope to a machine they
control without a hosted approval service. Origin private material stays
inside AuthorityWorker.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/rekey-inventory-20260910/Rekey功能清单与Agent任务优先级.xlsx
+++ b/outputs/rekey-inventory-20260910/Rekey功能清单与Agent任务优先级.xlsx
@@ -549,7 +549,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10 可执行清单已收口：P0/P1/P2与KEY-06、APR-08本机端完成；远程审批与其余35项P3待前提。维护与明确排除项保留原边界。</t>
+          <t>2026-09-10 可执行清单已收口：P0/P1/P2与KEY-06、APR-08本机端与challenge来源认证完成；托管远程审批服务与其余35项P3待前提。维护与明确排除项保留原边界。</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>本机独立审批端已验收</t>
+          <t>来源认证已验收；托管远程服务未实现</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>用户选择本人审批、先仅本机独立端。单人一次性review/sign已完成；使用步骤见 docs/user-guide.md#local-independent-approval-endpoint。远程服务与来源认证仍未实现。</t>
+          <t>本人审批、本机独立端与origin信封已验收。prepare返回 Broker 签名信封；rekey approval origin 钉扎公钥；rekey-approval-sign 要求 --origin-key。使用步骤见 docs/user-guide.md#local-independent-approval-endpoint。托管/公网远程审批服务仍未实现。</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -2220,12 +2220,13 @@
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>本机最小规格已实现</t>
+          <t>本机签发与来源认证已实现；托管远程服务未实现</t>
         </is>
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>docs/superpowers/specs/2026-09-10-local-approval-endpoint.md</t>
+          <t>docs/superpowers/specs/2026-09-10-local-approval-endpoint.md
+docs/superpowers/specs/2026-09-10-approval-origin-authentication.md</t>
         </is>
       </c>
       <c r="M24" s="11" t="inlineStr">
@@ -2236,7 +2237,9 @@
       <c r="N24" s="9" t="inlineStr">
         <is>
           <t>crates/rekey-policy/src/bin/rekey-approval-sign.rs
-scripts/test-approval-signer-live.py</t>
+scripts/test-approval-signer-live.py
+crates/rekey-vault/src/crypto/approval_origin.rs
+crates/rekey-policy/src/signed.rs</t>
         </is>
       </c>
       <c r="O24" s="9" t="inlineStr">
@@ -2253,7 +2256,7 @@
       </c>
       <c r="Q24" s="10" t="inlineStr">
         <is>
-          <t>outputs/rekey-apr08-20260910：5项签发测试、6项Broker合同通过；真实Broker接受，正文/会话错配及重放拒绝，仅1次TLS请求。check/clippy通过。challenge无来源签名；需操作者可信转交，合并前人审。 本机使用步骤已写入 docs/user-guide.md#local-independent-approval-endpoint。</t>
+          <t>outputs/rekey-apr08-20260910：签发测试、Broker合同与来源认证通过；未签名/错origin/篡改challenge拒绝。cargo test --workspace 0 failed。信封认证 Broker challenge 字节，不是托管远程审批服务。合并前人审。</t>
         </is>
       </c>
     </row>
@@ -15132,7 +15135,7 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>P0/P1、BAK-06与7项P2均已验收；APR-08本机独立端已验收，远程服务仍进行中；KEY-06完成不可追溯撤销研究。其余35项P3待场景/部署前提，不整批实现。</t>
+          <t>P0/P1、BAK-06与7项P2均已验收；APR-08本机独立端与challenge来源认证已验收，托管远程审批服务仍未实现；KEY-06完成不可追溯撤销研究。其余35项P3待场景/部署前提，不整批实现。</t>
         </is>
       </c>
     </row>
@@ -15240,7 +15243,7 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>可执行项已做完。APR-08本机review/sign完成，远程范围保持进行中；KEY-06研究完成。另35项P3待场景/部署前提，不得当作本轮实施授权。</t>
+          <t>可执行项已做完。APR-08本机review/sign与origin信封完成，托管远程服务保持未实现；KEY-06研究完成。另35项P3待场景/部署前提，不得当作本轮实施授权。</t>
         </is>
       </c>
     </row>
@@ -15396,7 +15399,7 @@
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>7项P2真实进程/协议专项已通过；GitHub静态/在线issuer两run成功并已删除临时repo。Keycloak源码反射修复后二审、6项合同测试与主工作区live复跑通过；最终cargo test --workspace、check、clippy、格式、机械契约与CLI依赖检查均通过，见outputs/rekey-p2-progress-20260910的verified/final日志。 APR-08：5项签发测试、6项Broker合同与真实执行验收通过；错配/过期/重放拒绝。本机使用步骤已写入 user-guide。</t>
+          <t>7项P2真实进程/协议专项已通过；GitHub静态/在线issuer两run成功并已删除临时repo。Keycloak源码反射修复后二审、6项合同测试与主工作区live复跑通过；最终cargo test --workspace、check、clippy、格式、机械契约与CLI依赖检查均通过，见outputs/rekey-p2-progress-20260910的verified/final日志。 APR-08：5项签发测试、6项Broker合同与真实执行验收通过；错配/过期/重放拒绝。本机使用步骤已写入 user-guide。 APR-08来源认证：origin密钥由解锁VRK派生并在AuthorityWorker内签名；prepare返回信封；signer要求--origin-key。</t>
         </is>
       </c>
     </row>

</xml_diff>